<commit_message>
added share button; removed ambiguous metaphor
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B982CFAC-8B79-4B4B-87B6-D6BFDAA3FD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC29A64-B7BB-4DA7-8EBE-BFB3B7612FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="35">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -133,6 +133,15 @@
   </si>
   <si>
     <t>Tag</t>
+  </si>
+  <si>
+    <t>five-second-rule-explored</t>
+  </si>
+  <si>
+    <t>Numpy</t>
+  </si>
+  <si>
+    <t>Germs</t>
   </si>
 </sst>
 </file>
@@ -208,8 +217,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B16" totalsRowShown="0">
-  <autoFilter ref="A1:B16" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B19" totalsRowShown="0">
+  <autoFilter ref="A1:B19" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B16">
     <sortCondition ref="A1:A16"/>
   </sortState>
@@ -222,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B24" totalsRowShown="0">
-  <autoFilter ref="A1:B24" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B28" totalsRowShown="0">
+  <autoFilter ref="A1:B28" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B24">
     <sortCondition ref="A1:A24"/>
   </sortState>
@@ -552,11 +561,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
@@ -694,6 +703,30 @@
         <v>10</v>
       </c>
     </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -704,11 +737,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -909,6 +942,38 @@
         <v>6</v>
       </c>
     </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
added cats/tags to xlsx for new ptow post
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC29A64-B7BB-4DA7-8EBE-BFB3B7612FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480DECD3-4679-4B4D-ABC8-445723A199E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="39">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>Germs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unique </t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>ptow-sympy-vs-numpy</t>
+  </si>
+  <si>
+    <t>SymPy</t>
   </si>
 </sst>
 </file>
@@ -177,14 +189,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -217,8 +235,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B19" totalsRowShown="0">
-  <autoFilter ref="A1:B19" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B21" totalsRowShown="0">
+  <autoFilter ref="A1:B21" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B16">
     <sortCondition ref="A1:A16"/>
   </sortState>
@@ -231,14 +249,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B28" totalsRowShown="0">
-  <autoFilter ref="A1:B28" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B24">
-    <sortCondition ref="A1:A24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C31" totalsRowShown="0">
+  <autoFilter ref="A1:C31" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B28">
+    <sortCondition ref="B2:B28"/>
   </sortState>
-  <tableColumns count="2">
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
-    <tableColumn id="2" xr3:uid="{9FA29049-8E81-4079-9D9A-737CCB3015ED}" name="Post" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{9FA29049-8E81-4079-9D9A-737CCB3015ED}" name="Post" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{6B53B531-8A8E-4A4C-9C68-6C5572A0BA20}" name="Unique " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -561,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -727,6 +746,22 @@
         <v>32</v>
       </c>
     </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -737,16 +772,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -756,59 +792,68 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>32</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>3</v>
@@ -816,7 +861,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>3</v>
@@ -824,85 +869,88 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -910,68 +958,104 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>33</v>
-      </c>
       <c r="B26" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>4</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>32</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added pwot for // and %
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480DECD3-4679-4B4D-ABC8-445723A199E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3EA6AA-14F7-46EE-9352-BBB88C698DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="44">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -154,6 +154,21 @@
   </si>
   <si>
     <t>SymPy</t>
+  </si>
+  <si>
+    <t>ptow-integer-division-and-modulus</t>
+  </si>
+  <si>
+    <t>Integer Division</t>
+  </si>
+  <si>
+    <t>Modulus</t>
+  </si>
+  <si>
+    <t>Operators</t>
+  </si>
+  <si>
+    <t>Numeric Parsing</t>
   </si>
 </sst>
 </file>
@@ -191,10 +206,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -235,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B21" totalsRowShown="0">
-  <autoFilter ref="A1:B21" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B23" totalsRowShown="0">
+  <autoFilter ref="A1:B23" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B16">
     <sortCondition ref="A1:A16"/>
   </sortState>
@@ -249,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C31" totalsRowShown="0">
-  <autoFilter ref="A1:C31" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C36" totalsRowShown="0">
+  <autoFilter ref="A1:C36" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B28">
     <sortCondition ref="B2:B28"/>
   </sortState>
@@ -580,11 +595,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
@@ -762,6 +777,22 @@
         <v>37</v>
       </c>
     </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -772,12 +803,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -785,144 +816,143 @@
     <col min="13" max="13" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -930,7 +960,7 @@
       <c r="A17" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>0</v>
       </c>
     </row>
@@ -938,7 +968,7 @@
       <c r="A18" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>0</v>
       </c>
     </row>
@@ -946,7 +976,7 @@
       <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>0</v>
       </c>
     </row>
@@ -954,7 +984,7 @@
       <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>0</v>
       </c>
     </row>
@@ -962,10 +992,10 @@
       <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -973,7 +1003,7 @@
       <c r="A22" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>9</v>
       </c>
     </row>
@@ -981,10 +1011,10 @@
       <c r="A23" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -992,10 +1022,10 @@
       <c r="A24" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1003,7 +1033,7 @@
       <c r="A25" t="s">
         <v>16</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1011,7 +1041,7 @@
       <c r="A26" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1019,7 +1049,7 @@
       <c r="A27" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1027,7 +1057,7 @@
       <c r="A28" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1035,7 +1065,7 @@
       <c r="A29" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1043,7 +1073,7 @@
       <c r="A30" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1051,10 +1081,53 @@
       <c r="A31" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added post: How AI Turns Meaning into Math
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F64F29B-8F2E-4F00-878B-B2D3B541C256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{554E3294-75A9-4092-8F8A-1ADECEDA6BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="56">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -174,10 +174,37 @@
     <t>how-ai-reads-code</t>
   </si>
   <si>
-    <t>Code Interpretation</t>
-  </si>
-  <si>
     <t>Large Language Models</t>
+  </si>
+  <si>
+    <t>how-ai-turns-meaning-into-math</t>
+  </si>
+  <si>
+    <t>Mathematics</t>
+  </si>
+  <si>
+    <t>Embeddings</t>
+  </si>
+  <si>
+    <t>MATLAB</t>
+  </si>
+  <si>
+    <t>Vectors</t>
+  </si>
+  <si>
+    <t>AI Interpretation</t>
+  </si>
+  <si>
+    <t>Linear Algebra</t>
+  </si>
+  <si>
+    <t>Neural Geometry</t>
+  </si>
+  <si>
+    <t>Mathematical Semantics</t>
+  </si>
+  <si>
+    <t>Code Semantics</t>
   </si>
 </sst>
 </file>
@@ -213,11 +240,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -258,8 +286,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B25" totalsRowShown="0">
-  <autoFilter ref="A1:B25" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:B28" totalsRowShown="0">
+  <autoFilter ref="A1:B28" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B25">
     <sortCondition ref="A1:A25"/>
   </sortState>
@@ -272,10 +300,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C38" totalsRowShown="0">
-  <autoFilter ref="A1:C38" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B28">
-    <sortCondition ref="B2:B28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C45" totalsRowShown="0">
+  <autoFilter ref="A1:C45" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C45">
+    <sortCondition ref="B2:B45"/>
+    <sortCondition ref="A2:A45"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
@@ -603,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -817,6 +846,30 @@
         <v>39</v>
       </c>
     </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -827,10 +880,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.42578125" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -888,93 +941,96 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>44</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>3</v>
+        <v>54</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>3</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>6</v>
+        <v>53</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>36</v>
@@ -982,115 +1038,112 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B28" t="s">
-        <v>10</v>
+        <v>39</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1098,80 +1151,139 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>37</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>44</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>0</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>8</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>15</v>
+      </c>
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
renamed posts to align with series
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{554E3294-75A9-4092-8F8A-1ADECEDA6BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6FA16D-602A-4BB1-9FD9-2255C797B2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="59">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -205,6 +205,15 @@
   </si>
   <si>
     <t>Code Semantics</t>
+  </si>
+  <si>
+    <t>LLM</t>
+  </si>
+  <si>
+    <t>how-large-languag-models-read-code</t>
+  </si>
+  <si>
+    <t>how-large-languag-models-think</t>
   </si>
 </sst>
 </file>
@@ -240,12 +249,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -300,11 +308,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C45" totalsRowShown="0">
-  <autoFilter ref="A1:C45" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C45">
-    <sortCondition ref="B2:B45"/>
-    <sortCondition ref="A2:A45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:C47" totalsRowShown="0">
+  <autoFilter ref="A1:C47" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C47">
+    <sortCondition ref="B2:B47"/>
+    <sortCondition ref="A2:A47"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
@@ -880,7 +888,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -944,7 +952,7 @@
         <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>36</v>
@@ -955,7 +963,7 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -963,82 +971,79 @@
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>36</v>
+        <v>52</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>46</v>
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>3</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
         <v>3</v>
@@ -1046,15 +1051,18 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
         <v>3</v>
       </c>
+      <c r="C18" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
         <v>3</v>
@@ -1062,7 +1070,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
         <v>3</v>
@@ -1070,7 +1078,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
         <v>3</v>
@@ -1078,23 +1086,23 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
@@ -1102,45 +1110,42 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>6</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
@@ -1148,18 +1153,21 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
       </c>
+      <c r="C30" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1167,39 +1175,39 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
         <v>0</v>
@@ -1207,7 +1215,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B37" t="s">
         <v>0</v>
@@ -1215,29 +1223,26 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B38" t="s">
         <v>0</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>36</v>
@@ -1245,34 +1250,37 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B42" t="s">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
         <v>10</v>
       </c>
+      <c r="C43" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B44" t="s">
         <v>10</v>
@@ -1280,9 +1288,25 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>4</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B47" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New post: LLM context windows
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE1424A-A46C-4A1F-B7E5-BD71F4962DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA2AAD7-66E1-4314-B39B-061EB8CF4DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="66">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -221,6 +221,21 @@
   </si>
   <si>
     <t>Should You Walk or Run in the Rain? The Puzzle That Sparked a Passion</t>
+  </si>
+  <si>
+    <t>how-large-language-models-handle-context-windows</t>
+  </si>
+  <si>
+    <t>How Large Language Models (LLMs) Handle Context Windows: The Memory That Isn't Memory</t>
+  </si>
+  <si>
+    <t>attention mechanisms</t>
+  </si>
+  <si>
+    <t>context windows</t>
+  </si>
+  <si>
+    <t>transformers</t>
   </si>
 </sst>
 </file>
@@ -263,9 +278,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -318,11 +334,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B49" totalsRowShown="0">
-  <autoFilter ref="A1:B49" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B49">
-    <sortCondition ref="B2:B49"/>
-    <sortCondition ref="A2:A49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B54" totalsRowShown="0">
+  <autoFilter ref="A1:B54" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B54">
+    <sortCondition ref="B2:B54"/>
+    <sortCondition ref="A2:A54"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
@@ -653,7 +669,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="85.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -807,6 +823,17 @@
         <v>53</v>
       </c>
     </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
     </row>
@@ -826,11 +853,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -882,40 +909,40 @@
       <c r="A6" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>40</v>
+      <c r="B6" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
+        <v>63</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
+        <v>64</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
-      <c r="B9" t="s">
-        <v>40</v>
+      <c r="B9" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>40</v>
+        <v>65</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -923,119 +950,119 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -1043,39 +1070,39 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -1083,150 +1110,190 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B38" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B40" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>25</v>
+      </c>
+      <c r="B52" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>32</v>
+      </c>
+      <c r="B53" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>3</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B54" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New Post: Birthday Paradox
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADA2327F-57B1-4241-B6FB-2F0D6EDEC2CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01228228-9909-4411-AEA3-EEE6CB0FCDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19215" yWindow="375" windowWidth="19410" windowHeight="15585" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="79">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -262,6 +262,18 @@
   </si>
   <si>
     <t>passwords</t>
+  </si>
+  <si>
+    <t>The Birthday Paradox in Production: When Random IDs Collide</t>
+  </si>
+  <si>
+    <t>birthday-paradox</t>
+  </si>
+  <si>
+    <t>databases</t>
+  </si>
+  <si>
+    <t>distributed-systems</t>
   </si>
 </sst>
 </file>
@@ -305,27 +317,13 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -339,6 +337,20 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -358,14 +370,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:C17" totalsRowShown="0">
-  <autoFilter ref="A1:C17" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:C18" totalsRowShown="0">
+  <autoFilter ref="A1:C18" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C17">
     <sortCondition ref="A2:A17"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{F23996D8-E038-415A-AB46-54564A371285}" name="Category"/>
-    <tableColumn id="2" xr3:uid="{39A3421C-15E2-433F-BE66-3D63EEDD4687}" name="Post" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{39A3421C-15E2-433F-BE66-3D63EEDD4687}" name="Post" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{C02648FB-67D5-4ADC-9EBC-5B72CAD5619A}" name="Title"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -373,15 +385,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B61" totalsRowShown="0">
-  <autoFilter ref="A1:B61" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B61">
-    <sortCondition ref="B2:B61"/>
-    <sortCondition ref="A2:A61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B66" totalsRowShown="0">
+  <autoFilter ref="A1:B66" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B66">
+    <sortCondition ref="B2:B66"/>
+    <sortCondition ref="A2:A66"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
-    <tableColumn id="2" xr3:uid="{9FA29049-8E81-4079-9D9A-737CCB3015ED}" name="Post" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{9FA29049-8E81-4079-9D9A-737CCB3015ED}" name="Post" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -704,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
@@ -734,7 +746,7 @@
       <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" t="s">
@@ -745,7 +757,7 @@
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
@@ -756,7 +768,7 @@
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C4" t="s">
@@ -767,7 +779,7 @@
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C5" t="s">
@@ -778,7 +790,7 @@
       <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C6" t="s">
@@ -789,7 +801,7 @@
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
@@ -800,7 +812,7 @@
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C8" t="s">
@@ -811,7 +823,7 @@
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C9" t="s">
@@ -822,7 +834,7 @@
       <c r="A10" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C10" t="s">
@@ -833,7 +845,7 @@
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
@@ -844,7 +856,7 @@
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C12" t="s">
@@ -855,7 +867,7 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
@@ -866,7 +878,7 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>68</v>
       </c>
       <c r="C14" t="s">
@@ -877,7 +889,7 @@
       <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C15" t="s">
@@ -888,7 +900,7 @@
       <c r="A16" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C16" t="s">
@@ -899,11 +911,22 @@
       <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C17" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -916,7 +939,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -938,106 +961,106 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
+        <v>70</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
+        <v>77</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
+        <v>78</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>68</v>
+        <v>34</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>68</v>
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>68</v>
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1045,23 +1068,23 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -1069,15 +1092,15 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -1085,71 +1108,71 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -1157,119 +1180,119 @@
         <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="B35" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="B36" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -1277,39 +1300,39 @@
         <v>3</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B48" t="s">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -1317,95 +1340,95 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>32</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>65</v>
+        <v>36</v>
+      </c>
+      <c r="B50" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B52" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B53" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B55" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B59" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B60" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -1413,6 +1436,46 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>37</v>
+      </c>
+      <c r="B62" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>16</v>
+      </c>
+      <c r="B63" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>25</v>
+      </c>
+      <c r="B64" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>3</v>
+      </c>
+      <c r="B66" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new blog post: edmund fitzgerald
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01228228-9909-4411-AEA3-EEE6CB0FCDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3820FED-D8D1-4035-A616-2309B2CCB6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="82">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -274,6 +274,15 @@
   </si>
   <si>
     <t>distributed-systems</t>
+  </si>
+  <si>
+    <t>edmund-fitzgerald</t>
+  </si>
+  <si>
+    <t>The Wreck of the Edmund Fitzgerald: Modeling Decomposition in Extreme Environments</t>
+  </si>
+  <si>
+    <t>biology</t>
   </si>
 </sst>
 </file>
@@ -370,8 +379,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:C18" totalsRowShown="0">
-  <autoFilter ref="A1:C18" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:C19" totalsRowShown="0">
+  <autoFilter ref="A1:C19" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C17">
     <sortCondition ref="A2:A17"/>
   </sortState>
@@ -385,8 +394,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B66" totalsRowShown="0">
-  <autoFilter ref="A1:B66" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B70" totalsRowShown="0">
+  <autoFilter ref="A1:B70" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B66">
     <sortCondition ref="B2:B66"/>
     <sortCondition ref="A2:A66"/>
@@ -716,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
@@ -929,6 +938,17 @@
         <v>75</v>
       </c>
     </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -939,7 +959,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A5A7A2-6C88-4B5B-9CA2-1FC13B12127A}">
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -1479,6 +1499,38 @@
         <v>5</v>
       </c>
     </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>3</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>32</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>37</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated about material to match Linkedin profile
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449F5076-1023-418C-B949-D768AC77C3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA71631-E64A-4B44-963C-9D3B4359D07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -454,8 +454,8 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}" name="Table3" displayName="Table3" ref="A1:B94" totalsRowShown="0">
   <autoFilter ref="A1:B94" xr:uid="{07C3CC26-95B6-4B44-8B92-969D553E6E58}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B84">
-    <sortCondition ref="B1:B84"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B94">
+    <sortCondition ref="B2:B94"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{7A38640D-FB54-4A3A-B307-2BCDCDCF5A4D}" name="Tag"/>
@@ -1649,168 +1649,168 @@
       <c r="A74" t="s">
         <v>17</v>
       </c>
-      <c r="B74" t="s">
-        <v>4</v>
+      <c r="B74" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>23</v>
-      </c>
-      <c r="B75" t="s">
-        <v>4</v>
+        <v>94</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>27</v>
-      </c>
-      <c r="B76" t="s">
-        <v>4</v>
+        <v>90</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>33</v>
-      </c>
-      <c r="B77" t="s">
-        <v>4</v>
+        <v>95</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>24</v>
-      </c>
-      <c r="B78" t="s">
-        <v>39</v>
+        <v>96</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>3</v>
-      </c>
-      <c r="B79" t="s">
-        <v>39</v>
+        <v>32</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>36</v>
-      </c>
-      <c r="B80" t="s">
-        <v>39</v>
+        <v>97</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>16</v>
-      </c>
-      <c r="B81" t="s">
-        <v>5</v>
+        <v>98</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>25</v>
-      </c>
-      <c r="B82" t="s">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>30</v>
-      </c>
-      <c r="B83" t="s">
-        <v>5</v>
+        <v>100</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B84" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>17</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>85</v>
+        <v>23</v>
+      </c>
+      <c r="B85" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>94</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>85</v>
+        <v>27</v>
+      </c>
+      <c r="B86" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>90</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>85</v>
+        <v>33</v>
+      </c>
+      <c r="B87" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>95</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>85</v>
+        <v>24</v>
+      </c>
+      <c r="B88" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>96</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>85</v>
+        <v>3</v>
+      </c>
+      <c r="B89" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>32</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>85</v>
+        <v>36</v>
+      </c>
+      <c r="B90" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>97</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>85</v>
+        <v>16</v>
+      </c>
+      <c r="B91" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>98</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>85</v>
+        <v>25</v>
+      </c>
+      <c r="B92" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>99</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>85</v>
+        <v>30</v>
+      </c>
+      <c r="B93" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>100</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>85</v>
+        <v>3</v>
+      </c>
+      <c r="B94" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed polyfill.io cdn reference
</commit_message>
<xml_diff>
--- a/data/CategoriesAndTags.xlsx
+++ b/data/CategoriesAndTags.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA71631-E64A-4B44-963C-9D3B4359D07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B2EE9B-2C18-470E-85D5-7AF0C96244D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="3630" yWindow="3630" windowWidth="43200" windowHeight="11235" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="102">
   <si>
     <t>rain-paradox</t>
   </si>
@@ -340,13 +340,16 @@
   </si>
   <si>
     <t>top-p</t>
+  </si>
+  <si>
+    <t>URL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,6 +359,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -378,31 +389,38 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFF0000"/>
+        <color auto="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -422,6 +440,20 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -436,16 +468,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:C22" totalsRowShown="0">
-  <autoFilter ref="A1:C22" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:D22" totalsRowShown="0">
+  <autoFilter ref="A1:D22" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C22">
     <sortCondition ref="A2:A22"/>
     <sortCondition ref="B2:B22"/>
   </sortState>
-  <tableColumns count="3">
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{F23996D8-E038-415A-AB46-54564A371285}" name="Category"/>
-    <tableColumn id="2" xr3:uid="{39A3421C-15E2-433F-BE66-3D63EEDD4687}" name="Post" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{39A3421C-15E2-433F-BE66-3D63EEDD4687}" name="Post" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{C02648FB-67D5-4ADC-9EBC-5B72CAD5619A}" name="Title"/>
+    <tableColumn id="4" xr3:uid="{98EF9C75-81CD-4D8A-B580-7C33356E2373}" name="URL" dataDxfId="0">
+      <calculatedColumnFormula>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -782,22 +817,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEE28CF5-D7ED-41A9-98E3-4DEECEEA1CE1}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="85.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="85.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -807,8 +839,11 @@
       <c r="C1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -818,8 +853,12 @@
       <c r="C2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/discrete-math-in-large-language-models</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -829,8 +868,12 @@
       <c r="C3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-language-models-handle-context-windows</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -840,8 +883,12 @@
       <c r="C4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-language-models-know-things-they-were-never-taught</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -851,8 +898,12 @@
       <c r="C5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-languag-models-learn</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -862,8 +913,12 @@
       <c r="C6" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-languag-models-read-code</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -873,8 +928,12 @@
       <c r="C7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-languag-models-think</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -884,8 +943,12 @@
       <c r="C8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-languag-models-tokenize-text</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -895,8 +958,12 @@
       <c r="C9" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/temperature-top-p-creativity-knobs</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -906,8 +973,12 @@
       <c r="C10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/birthday-paradox</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -917,8 +988,12 @@
       <c r="C11" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/edmund-fitzgerald</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -928,8 +1003,12 @@
       <c r="C12" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/five-second-rule</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -939,8 +1018,12 @@
       <c r="C13" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/meeting-diet</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -950,8 +1033,12 @@
       <c r="C14" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/rain-paradox</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -961,8 +1048,12 @@
       <c r="C15" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/safe-distance-in-traffic</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -972,8 +1063,12 @@
       <c r="C16" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/thermo-water-energy-balance</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -983,8 +1078,12 @@
       <c r="C17" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/three-d-packing</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -994,8 +1093,12 @@
       <c r="C18" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/hash-collisions</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1005,8 +1108,12 @@
       <c r="C19" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/tfp-chatgpt</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -1016,8 +1123,12 @@
       <c r="C20" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/python-dispatch-maps</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -1027,8 +1138,12 @@
       <c r="C21" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/python-integer-division-and-modulus</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -1037,6 +1152,10 @@
       </c>
       <c r="C22" t="s">
         <v>44</v>
+      </c>
+      <c r="D22" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/python-sympy-vs-numpy</v>
       </c>
     </row>
   </sheetData>
@@ -1113,7 +1232,7 @@
       <c r="A7" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1121,7 +1240,7 @@
       <c r="A8" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1129,7 +1248,7 @@
       <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1137,7 +1256,7 @@
       <c r="A10" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1145,7 +1264,7 @@
       <c r="A11" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1153,7 +1272,7 @@
       <c r="A12" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1161,7 +1280,7 @@
       <c r="A13" t="s">
         <v>89</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1305,7 +1424,7 @@
       <c r="A31" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1313,7 +1432,7 @@
       <c r="A32" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1321,7 +1440,7 @@
       <c r="A33" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1329,7 +1448,7 @@
       <c r="A34" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1337,7 +1456,7 @@
       <c r="A35" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1633,7 +1752,7 @@
       <c r="A72" t="s">
         <v>93</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1641,7 +1760,7 @@
       <c r="A73" t="s">
         <v>3</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1649,7 +1768,7 @@
       <c r="A74" t="s">
         <v>17</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1657,7 +1776,7 @@
       <c r="A75" t="s">
         <v>94</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1665,7 +1784,7 @@
       <c r="A76" t="s">
         <v>90</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1673,7 +1792,7 @@
       <c r="A77" t="s">
         <v>95</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1681,7 +1800,7 @@
       <c r="A78" t="s">
         <v>96</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1689,7 +1808,7 @@
       <c r="A79" t="s">
         <v>32</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1697,7 +1816,7 @@
       <c r="A80" t="s">
         <v>97</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1705,7 +1824,7 @@
       <c r="A81" t="s">
         <v>98</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1713,7 +1832,7 @@
       <c r="A82" t="s">
         <v>99</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1721,7 +1840,7 @@
       <c r="A83" t="s">
         <v>100</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>